<commit_message>
Updated transition dataset prep
</commit_message>
<xml_diff>
--- a/tools/scenario_specifications.xlsx
+++ b/tools/scenario_specifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A5DE42-E428-4461-A56B-3370D973DB50}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F00BB420-DF05-4C8F-9559-454B6133380D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="6480" activeTab="1" xr2:uid="{89DA8B81-9916-4047-9C32-2B28CB7C6979}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
   <si>
     <t>Scenario_ID</t>
   </si>
@@ -70,10 +70,34 @@
     <t>Build_zone</t>
   </si>
   <si>
-    <t>Ref_Urban</t>
-  </si>
-  <si>
     <t>Econ_scenario</t>
+  </si>
+  <si>
+    <t>Ecolo_Urban</t>
+  </si>
+  <si>
+    <t>Ref_Peri_urban</t>
+  </si>
+  <si>
+    <t>Ecolo_Central</t>
+  </si>
+  <si>
+    <t>Ref_Central</t>
+  </si>
+  <si>
+    <t>Combined_Urban</t>
+  </si>
+  <si>
+    <t>Climate_RCP</t>
+  </si>
+  <si>
+    <t>RCP45</t>
+  </si>
+  <si>
+    <t>RCP26</t>
+  </si>
+  <si>
+    <t>RCP85</t>
   </si>
 </sst>
 </file>
@@ -525,14 +549,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32ADE76A-93A5-421C-9EF7-AF707F3C674A}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -540,10 +565,13 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -551,10 +579,13 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -562,10 +593,13 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -573,10 +607,13 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -584,10 +621,13 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -595,7 +635,10 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated process of simulation transition rates prep
</commit_message>
<xml_diff>
--- a/tools/scenario_specifications.xlsx
+++ b/tools/scenario_specifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B055C4-9956-41C4-A516-92950562710F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C097655F-DE68-4114-B6E6-076A409304D3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="6480" xr2:uid="{89DA8B81-9916-4047-9C32-2B28CB7C6979}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="45">
   <si>
     <t>Scenario_ID</t>
   </si>
@@ -112,9 +112,6 @@
     <t>Data/Spat_prob_perturb_layers/Bulding_zones/BZ_raster.grd</t>
   </si>
   <si>
-    <t>Data/Spat_prob_perturb_layers/Municipality_typology/Muni_type_raster.grd"</t>
-  </si>
-  <si>
     <t>Urban_migration</t>
   </si>
   <si>
@@ -124,7 +121,46 @@
     <t>Mountain_development</t>
   </si>
   <si>
-    <t>2020, 2025, 2030</t>
+    <t>2020, 2025, 2030, 2035, 2040, 2045, 2050,2055, 2060</t>
+  </si>
+  <si>
+    <t>Data/Spat_prob_perturb_layers/Municipality_typology/Muni_type_raster.grd</t>
+  </si>
+  <si>
+    <t>Prob_perturb_threshold</t>
+  </si>
+  <si>
+    <t>Agri_abandonment</t>
+  </si>
+  <si>
+    <t>Agri_maintenance</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Shrubland, Open_Forest</t>
+  </si>
+  <si>
+    <t>Shrubland, Open_Forest, Grassland</t>
+  </si>
+  <si>
+    <t>Urban, Static</t>
+  </si>
+  <si>
+    <t>Urban, Int_Ag, Open_Forest, Grassland, Perm_Crops, Alp_Past</t>
+  </si>
+  <si>
+    <t>Spatial_zoning</t>
+  </si>
+  <si>
+    <t>Param_adjust</t>
+  </si>
+  <si>
+    <t>Intervention_type</t>
+  </si>
+  <si>
+    <t>Prob_adjust</t>
   </si>
 </sst>
 </file>
@@ -477,15 +513,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{563B5FA0-3F45-4EC9-BC2A-659950A4E6A9}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="2" max="3" width="23.85546875" customWidth="1"/>
+    <col min="4" max="4" width="37.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -493,183 +530,381 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8" t="s">
         <v>32</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="F9">
+        <v>5</v>
+      </c>
+      <c r="G9" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" t="s">
         <v>23</v>
       </c>
-      <c r="E5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11">
+        <v>5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12">
+        <v>5</v>
+      </c>
+      <c r="G12" t="s">
         <v>32</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" t="s">
         <v>23</v>
       </c>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="F13">
+        <v>5</v>
+      </c>
+      <c r="G13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14">
+        <v>5</v>
+      </c>
+      <c r="G14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15">
+        <v>5</v>
+      </c>
+      <c r="G15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" t="s">
-        <v>28</v>
+      <c r="B17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17">
+        <v>5</v>
+      </c>
+      <c r="G17" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>